<commit_message>
Okakura Kakuzō everywhere (family name first, with the macron): thoughts, calendar, and glossary masters, rebuilt JSON; change log in exports/
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/calendar.xlsx
+++ b/content/calendar.xlsx
@@ -2250,7 +2250,7 @@
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. II</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. II</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. III</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. III</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. V</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. V</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
@@ -12340,7 +12340,7 @@
       </c>
       <c r="E273" s="9" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. III</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. III</t>
         </is>
       </c>
       <c r="F273" s="9" t="inlineStr">
@@ -13322,7 +13322,7 @@
       </c>
       <c r="E295" s="5" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. IV</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. IV</t>
         </is>
       </c>
       <c r="F295" s="5" t="inlineStr">
@@ -14298,7 +14298,7 @@
       </c>
       <c r="E317" s="5" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. I</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. I</t>
         </is>
       </c>
       <c r="F317" s="5" t="inlineStr">
@@ -17269,7 +17269,7 @@
       </c>
       <c r="E384" s="7" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. I</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. I</t>
         </is>
       </c>
       <c r="F384" s="7" t="inlineStr">
@@ -19000,7 +19000,7 @@
       </c>
       <c r="E423" s="9" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. V</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. V</t>
         </is>
       </c>
       <c r="F423" s="9" t="inlineStr">
@@ -19626,7 +19626,7 @@
       </c>
       <c r="E437" s="5" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. III</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. III</t>
         </is>
       </c>
       <c r="F437" s="5" t="inlineStr">
@@ -20682,7 +20682,7 @@
       </c>
       <c r="E461" s="7" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. III</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. III</t>
         </is>
       </c>
       <c r="F461" s="7" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="E494" s="5" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. I</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. I</t>
         </is>
       </c>
       <c r="F494" s="5" t="inlineStr">
@@ -22775,7 +22775,7 @@
       </c>
       <c r="E508" s="5" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. VII</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. VII</t>
         </is>
       </c>
       <c r="F508" s="5" t="inlineStr">
@@ -25439,7 +25439,7 @@
       </c>
       <c r="E568" s="5" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. IV</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. IV</t>
         </is>
       </c>
       <c r="F568" s="5" t="inlineStr">
@@ -25967,7 +25967,7 @@
       </c>
       <c r="E580" s="7" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. I</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. I</t>
         </is>
       </c>
       <c r="F580" s="7" t="inlineStr">
@@ -27563,7 +27563,7 @@
       </c>
       <c r="E616" s="9" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. I</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. I</t>
         </is>
       </c>
       <c r="F616" s="9" t="inlineStr">
@@ -31694,7 +31694,7 @@
       </c>
       <c r="E709" s="5" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. III</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. III</t>
         </is>
       </c>
       <c r="F709" s="5" t="inlineStr">
@@ -32492,7 +32492,7 @@
       </c>
       <c r="E727" s="7" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. IV</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. IV</t>
         </is>
       </c>
       <c r="F727" s="7" t="inlineStr">
@@ -33468,7 +33468,7 @@
       </c>
       <c r="E749" s="9" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. I</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. I</t>
         </is>
       </c>
       <c r="F749" s="9" t="inlineStr">
@@ -33652,7 +33652,7 @@
       </c>
       <c r="E753" s="5" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura, The Book of Tea, ch. VI</t>
+          <t>Okakura Kakuzō, The Book of Tea, ch. VI</t>
         </is>
       </c>
       <c r="F753" s="5" t="inlineStr">

</xml_diff>